<commit_message>
chore: update dataset files and add memory usage analysis script for troubleshooting
</commit_message>
<xml_diff>
--- a/match_ingestion_summary.xlsx
+++ b/match_ingestion_summary.xlsx
@@ -532,10 +532,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3531</v>
+        <v>3532</v>
       </c>
       <c r="C5" t="n">
-        <v>2712</v>
+        <v>2713</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C6" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update T20 match data and ingestion summary parquet and excel files
</commit_message>
<xml_diff>
--- a/match_ingestion_summary.xlsx
+++ b/match_ingestion_summary.xlsx
@@ -509,10 +509,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="C4" t="n">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update dashboard timestamps, refresh match datasets, and ignore summary spreadsheet in git
</commit_message>
<xml_diff>
--- a/match_ingestion_summary.xlsx
+++ b/match_ingestion_summary.xlsx
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C6" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>

</xml_diff>